<commit_message>
M15 step 3 (awaiting owner's check): import of deliveries and sales since the starting day
The Deliveries and Sales sheets are checked whole, then replayed in the order
things happened in one transaction. Imported sales keep their own date and an
IMP- receipt number, go through no till, and a shortage is accepted and listed
as an exception. The writing of a sale moved into src/server/sale-write.ts so
the checkout, offline sync and the import share one writer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/kuchpos-import-template.xlsx
+++ b/public/templates/kuchpos-import-template.xlsx
@@ -45,12 +45,18 @@
     <t>7. In KuchPos, sign in as the admin, open Settings, then Import from Excel, and choose this file. You are shown what will be brought in, and every row that has a problem, before anything is saved.</t>
   </si>
   <si>
-    <t>8. Products, Customers and Stock are brought in first. Deliveries and Sales are brought in afterwards, in a second step.</t>
+    <t>8. Products, Customers and Stock are brought in first (step 2 on that page). Deliveries and Sales are brought in afterwards (step 3), in the order they happened. No date may be earlier than the day the records start.</t>
   </si>
   <si>
     <t>9. A product or customer that is already in KuchPos is left as it is, so the same file can be used again after adding more rows. Stock rows are different: once a product's starting stock is in, delete its row from the Stock sheet before using the file again.</t>
   </si>
   <si>
+    <t>10. A delivery (by its reference and supplier) or a sale (by its receipt number) can be brought in only once. For later deliveries and sales, use a file that holds only the new ones.</t>
+  </si>
+  <si>
+    <t>11. Money that customers paid back on their debts since the starting day is not in this workbook. After the import, record each one in KuchPos as a repayment on the customer's page.</t>
+  </si>
+  <si>
     <t>Product code *</t>
   </si>
   <si>
@@ -291,7 +297,7 @@
     <t>Hour:minute, 24-hour clock. Helps the report by hour.</t>
   </si>
   <si>
-    <t>Your own receipt or reference number.</t>
+    <t>Your own receipt or reference number, 16 characters at most. It is kept, with IMP- in front.</t>
   </si>
   <si>
     <t>In Naira: what one of this unit was sold for.</t>
@@ -300,7 +306,7 @@
     <t>In Naira. Fill it on the first row of the sale only.</t>
   </si>
   <si>
-    <t>Cash, or the name of one of the shop's other payment methods.</t>
+    <t>Cash, or the name of one of the shop's other payment methods. One way of paying for a sale; a part not paid goes under Amount on credit.</t>
   </si>
   <si>
     <t>Must be on the Customers sheet.</t>
@@ -465,6 +471,16 @@
         <v>9</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -488,108 +504,108 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -610,63 +626,63 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -686,58 +702,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -761,81 +777,81 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J2" s="5"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -850,13 +866,13 @@
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
@@ -864,101 +880,101 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>

</xml_diff>

<commit_message>
M16 (in progress): error log for owners, error screens, security checklist, speed test on a large shop
Also from the speed test: the six-month sales report no longer builds a date
formatter per sale or reads lines it does not need; a history import file is
limited to 6,000 rows. The database driver is held at the patched 3.4.7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/kuchpos-import-template.xlsx
+++ b/public/templates/kuchpos-import-template.xlsx
@@ -54,7 +54,10 @@
     <t>10. A delivery (by its reference and supplier) or a sale (by its receipt number) can be brought in only once. For later deliveries and sales, use a file that holds only the new ones.</t>
   </si>
   <si>
-    <t>11. Money that customers paid back on their debts since the starting day is not in this workbook. After the import, record each one in KuchPos as a repayment on the customer's page.</t>
+    <t>11. Deliveries and Sales together: at most 6,000 rows in one file. If you have more, make several files by date (a week or two each) and bring them in one after another, the earliest first.</t>
+  </si>
+  <si>
+    <t>12. Money that customers paid back on their debts since the starting day is not in this workbook. After the import, record each one in KuchPos as a repayment on the customer's page.</t>
   </si>
   <si>
     <t>Product code *</t>
@@ -481,6 +484,11 @@
         <v>11</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -504,108 +512,108 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>34</v>
-      </c>
       <c r="H3" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -626,63 +634,63 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5"/>
       <c r="B2" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -702,58 +710,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -777,81 +785,81 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J2" s="5"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -880,101 +888,101 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>

</xml_diff>

<commit_message>
C70 (awaiting owner's check): analysis on the home, customer and product pages; Sold by must be staff on import; less for managers
Home page: top 5 products, categories and customers for admins and owners.
Customer page: purchases, products and amounts over a period, with a chart.
Product page: sales as a line over time, buyers, and each sale.
Managers: no credit limits (nor credit over a limit), no purchase totals,
no Reports pages. Three new permissions carry it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/kuchpos-import-template.xlsx
+++ b/public/templates/kuchpos-import-template.xlsx
@@ -318,7 +318,7 @@
     <t>In Naira. Needs the customer. Fill it on the first row of the sale only.</t>
   </si>
   <si>
-    <t>A name, kept as a note.</t>
+    <t>The full name or username of a staff member, as on the Staff page; or leave empty.</t>
   </si>
   <si>
     <t>02/10/2026</t>
@@ -883,7 +883,7 @@
     <col min="9" max="9" width="30" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="20" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>